<commit_message>
Modifique los tamaños de la interfaz y arregle un problema del codigo con los 4to slot's
</commit_message>
<xml_diff>
--- a/datos/ACTIVIDADES_EJEMPLO_2025_salida.xlsx
+++ b/datos/ACTIVIDADES_EJEMPLO_2025_salida.xlsx
@@ -595,7 +595,7 @@
         <v>9</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G2" t="s">
         <v>10</v>
@@ -618,7 +618,7 @@
         <v>9</v>
       </c>
       <c r="F3" t="n">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G3" t="s">
         <v>11</v>
@@ -664,7 +664,7 @@
         <v>9</v>
       </c>
       <c r="F5" t="n">
-        <v>220</v>
+        <v>241</v>
       </c>
       <c r="G5" t="s">
         <v>13</v>
@@ -687,7 +687,7 @@
         <v>14</v>
       </c>
       <c r="F6" t="n">
-        <v>304</v>
+        <v>308</v>
       </c>
       <c r="G6" t="s">
         <v>15</v>
@@ -710,7 +710,7 @@
         <v>9</v>
       </c>
       <c r="F7" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="G7" t="s">
         <v>17</v>
@@ -733,7 +733,7 @@
         <v>9</v>
       </c>
       <c r="F8" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G8" t="s">
         <v>17</v>
@@ -756,7 +756,7 @@
         <v>9</v>
       </c>
       <c r="F9" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="G9" t="s">
         <v>17</v>
@@ -802,7 +802,7 @@
         <v>14</v>
       </c>
       <c r="F11" t="n">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="G11" t="s">
         <v>17</v>
@@ -825,7 +825,7 @@
         <v>9</v>
       </c>
       <c r="F12" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="G12" t="s">
         <v>18</v>
@@ -848,7 +848,7 @@
         <v>9</v>
       </c>
       <c r="F13" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="G13" t="s">
         <v>18</v>
@@ -871,7 +871,7 @@
         <v>9</v>
       </c>
       <c r="F14" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="G14" t="s">
         <v>18</v>
@@ -917,7 +917,7 @@
         <v>14</v>
       </c>
       <c r="F16" t="n">
-        <v>65</v>
+        <v>8</v>
       </c>
       <c r="G16" t="s">
         <v>18</v>
@@ -940,7 +940,7 @@
         <v>9</v>
       </c>
       <c r="F17" t="n">
-        <v>62</v>
+        <v>100</v>
       </c>
       <c r="G17" t="s">
         <v>19</v>
@@ -963,7 +963,7 @@
         <v>9</v>
       </c>
       <c r="F18" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="G18" t="s">
         <v>19</v>
@@ -1055,7 +1055,7 @@
         <v>14</v>
       </c>
       <c r="F22" t="n">
-        <v>1864</v>
+        <v>1870</v>
       </c>
       <c r="G22" t="s">
         <v>19</v>
@@ -1078,7 +1078,7 @@
         <v>14</v>
       </c>
       <c r="F23" t="n">
-        <v>1861</v>
+        <v>1873</v>
       </c>
       <c r="G23" t="s">
         <v>18</v>
@@ -1101,7 +1101,7 @@
         <v>14</v>
       </c>
       <c r="F24" t="n">
-        <v>1873</v>
+        <v>1848</v>
       </c>
       <c r="G24" t="s">
         <v>17</v>
@@ -1124,7 +1124,7 @@
         <v>9</v>
       </c>
       <c r="F25" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G25" t="s">
         <v>21</v>
@@ -1147,7 +1147,7 @@
         <v>9</v>
       </c>
       <c r="F26" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="G26" t="s">
         <v>22</v>
@@ -1170,7 +1170,7 @@
         <v>14</v>
       </c>
       <c r="F27" t="n">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="G27" t="s">
         <v>23</v>
@@ -1193,7 +1193,7 @@
         <v>14</v>
       </c>
       <c r="F28" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="G28" t="s">
         <v>24</v>
@@ -1216,7 +1216,7 @@
         <v>14</v>
       </c>
       <c r="F29" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G29" t="s">
         <v>21</v>
@@ -1239,7 +1239,7 @@
         <v>9</v>
       </c>
       <c r="F30" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="G30" t="s">
         <v>25</v>
@@ -1262,7 +1262,7 @@
         <v>9</v>
       </c>
       <c r="F31" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="G31" t="s">
         <v>21</v>
@@ -1285,7 +1285,7 @@
         <v>14</v>
       </c>
       <c r="F32" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="G32" t="s">
         <v>26</v>
@@ -1308,7 +1308,7 @@
         <v>14</v>
       </c>
       <c r="F33" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G33" t="s">
         <v>27</v>
@@ -1377,7 +1377,7 @@
         <v>14</v>
       </c>
       <c r="F36" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="G36" t="s">
         <v>21</v>
@@ -1423,7 +1423,7 @@
         <v>9</v>
       </c>
       <c r="F38" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="G38" t="s">
         <v>28</v>
@@ -1446,7 +1446,7 @@
         <v>9</v>
       </c>
       <c r="F39" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="G39" t="s">
         <v>30</v>
@@ -1469,7 +1469,7 @@
         <v>9</v>
       </c>
       <c r="F40" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G40" t="s">
         <v>30</v>
@@ -1538,7 +1538,7 @@
         <v>9</v>
       </c>
       <c r="F43" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G43" t="s">
         <v>31</v>
@@ -1561,7 +1561,7 @@
         <v>9</v>
       </c>
       <c r="F44" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G44" t="s">
         <v>31</v>
@@ -1607,7 +1607,7 @@
         <v>9</v>
       </c>
       <c r="F46" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="G46" t="s">
         <v>32</v>
@@ -1630,7 +1630,7 @@
         <v>9</v>
       </c>
       <c r="F47" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="G47" t="s">
         <v>32</v>
@@ -1653,7 +1653,7 @@
         <v>14</v>
       </c>
       <c r="F48" t="n">
-        <v>40</v>
+        <v>5</v>
       </c>
       <c r="G48" t="s">
         <v>32</v>
@@ -1676,7 +1676,7 @@
         <v>14</v>
       </c>
       <c r="F49" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="G49" t="s">
         <v>32</v>
@@ -1699,7 +1699,7 @@
         <v>9</v>
       </c>
       <c r="F50" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="G50" t="s">
         <v>33</v>
@@ -1722,7 +1722,7 @@
         <v>9</v>
       </c>
       <c r="F51" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="G51" t="s">
         <v>33</v>
@@ -1745,7 +1745,7 @@
         <v>14</v>
       </c>
       <c r="F52" t="n">
-        <v>40</v>
+        <v>18</v>
       </c>
       <c r="G52" t="s">
         <v>33</v>
@@ -1768,7 +1768,7 @@
         <v>14</v>
       </c>
       <c r="F53" t="n">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="G53" t="s">
         <v>33</v>
@@ -1791,7 +1791,7 @@
         <v>9</v>
       </c>
       <c r="F54" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="G54" t="s">
         <v>35</v>
@@ -1814,7 +1814,7 @@
         <v>9</v>
       </c>
       <c r="F55" t="n">
-        <v>278</v>
+        <v>283</v>
       </c>
       <c r="G55" t="s">
         <v>36</v>
@@ -1860,7 +1860,7 @@
         <v>9</v>
       </c>
       <c r="F57" t="n">
-        <v>247</v>
+        <v>221</v>
       </c>
       <c r="G57" t="s">
         <v>37</v>
@@ -1883,7 +1883,7 @@
         <v>14</v>
       </c>
       <c r="F58" t="n">
-        <v>372</v>
+        <v>312</v>
       </c>
       <c r="G58" t="s">
         <v>38</v>
@@ -1906,7 +1906,7 @@
         <v>9</v>
       </c>
       <c r="F59" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G59" t="s">
         <v>17</v>
@@ -1929,7 +1929,7 @@
         <v>9</v>
       </c>
       <c r="F60" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="G60" t="s">
         <v>17</v>
@@ -1952,7 +1952,7 @@
         <v>9</v>
       </c>
       <c r="F61" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G61" t="s">
         <v>17</v>
@@ -1998,7 +1998,7 @@
         <v>14</v>
       </c>
       <c r="F63" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="G63" t="s">
         <v>17</v>
@@ -2021,7 +2021,7 @@
         <v>9</v>
       </c>
       <c r="F64" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G64" t="s">
         <v>18</v>
@@ -2067,7 +2067,7 @@
         <v>9</v>
       </c>
       <c r="F66" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="G66" t="s">
         <v>18</v>
@@ -2113,7 +2113,7 @@
         <v>14</v>
       </c>
       <c r="F68" t="n">
-        <v>65</v>
+        <v>0</v>
       </c>
       <c r="G68" t="s">
         <v>18</v>
@@ -2136,7 +2136,7 @@
         <v>9</v>
       </c>
       <c r="F69" t="n">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="G69" t="s">
         <v>19</v>
@@ -2159,7 +2159,7 @@
         <v>9</v>
       </c>
       <c r="F70" t="n">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="G70" t="s">
         <v>19</v>
@@ -2251,7 +2251,7 @@
         <v>14</v>
       </c>
       <c r="F74" t="n">
-        <v>1885</v>
+        <v>1870</v>
       </c>
       <c r="G74" t="s">
         <v>19</v>
@@ -2274,7 +2274,7 @@
         <v>14</v>
       </c>
       <c r="F75" t="n">
-        <v>1900</v>
+        <v>1880</v>
       </c>
       <c r="G75" t="s">
         <v>18</v>
@@ -2297,7 +2297,7 @@
         <v>14</v>
       </c>
       <c r="F76" t="n">
-        <v>1888</v>
+        <v>1865</v>
       </c>
       <c r="G76" t="s">
         <v>17</v>
@@ -2320,7 +2320,7 @@
         <v>9</v>
       </c>
       <c r="F77" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="G77" t="s">
         <v>39</v>
@@ -2343,7 +2343,7 @@
         <v>9</v>
       </c>
       <c r="F78" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G78" t="s">
         <v>22</v>
@@ -2366,7 +2366,7 @@
         <v>14</v>
       </c>
       <c r="F79" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="G79" t="s">
         <v>40</v>
@@ -2389,7 +2389,7 @@
         <v>14</v>
       </c>
       <c r="F80" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="G80" t="s">
         <v>22</v>
@@ -2412,7 +2412,7 @@
         <v>9</v>
       </c>
       <c r="F81" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="G81" t="s">
         <v>41</v>
@@ -2435,7 +2435,7 @@
         <v>9</v>
       </c>
       <c r="F82" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G82" t="s">
         <v>39</v>
@@ -2458,7 +2458,7 @@
         <v>14</v>
       </c>
       <c r="F83" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="G83" t="s">
         <v>26</v>
@@ -2504,7 +2504,7 @@
         <v>9</v>
       </c>
       <c r="F85" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G85" t="s">
         <v>21</v>
@@ -2550,7 +2550,7 @@
         <v>9</v>
       </c>
       <c r="F87" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G87" t="s">
         <v>21</v>
@@ -2573,7 +2573,7 @@
         <v>14</v>
       </c>
       <c r="F88" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="G88" t="s">
         <v>21</v>
@@ -2619,7 +2619,7 @@
         <v>14</v>
       </c>
       <c r="F90" t="n">
-        <v>4</v>
+        <v>25</v>
       </c>
       <c r="G90" t="s">
         <v>21</v>
@@ -2642,7 +2642,7 @@
         <v>9</v>
       </c>
       <c r="F91" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="G91" t="s">
         <v>30</v>
@@ -2711,7 +2711,7 @@
         <v>14</v>
       </c>
       <c r="F94" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="G94" t="s">
         <v>30</v>
@@ -2780,7 +2780,7 @@
         <v>14</v>
       </c>
       <c r="F97" t="n">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="G97" t="s">
         <v>31</v>
@@ -2826,7 +2826,7 @@
         <v>9</v>
       </c>
       <c r="F99" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="G99" t="s">
         <v>32</v>
@@ -2872,7 +2872,7 @@
         <v>14</v>
       </c>
       <c r="F101" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="G101" t="s">
         <v>32</v>
@@ -2895,7 +2895,7 @@
         <v>9</v>
       </c>
       <c r="F102" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G102" t="s">
         <v>33</v>
@@ -2918,7 +2918,7 @@
         <v>9</v>
       </c>
       <c r="F103" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G103" t="s">
         <v>33</v>
@@ -2941,7 +2941,7 @@
         <v>14</v>
       </c>
       <c r="F104" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="G104" t="s">
         <v>33</v>
@@ -2964,7 +2964,7 @@
         <v>14</v>
       </c>
       <c r="F105" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="G105" t="s">
         <v>33</v>
@@ -2987,7 +2987,7 @@
         <v>9</v>
       </c>
       <c r="F106" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G106" t="s">
         <v>44</v>
@@ -3010,7 +3010,7 @@
         <v>9</v>
       </c>
       <c r="F107" t="n">
-        <v>291</v>
+        <v>315</v>
       </c>
       <c r="G107" t="s">
         <v>45</v>
@@ -3056,7 +3056,7 @@
         <v>9</v>
       </c>
       <c r="F109" t="n">
-        <v>231</v>
+        <v>249</v>
       </c>
       <c r="G109" t="s">
         <v>46</v>
@@ -3079,7 +3079,7 @@
         <v>14</v>
       </c>
       <c r="F110" t="n">
-        <v>274</v>
+        <v>197</v>
       </c>
       <c r="G110" t="s">
         <v>47</v>
@@ -3125,7 +3125,7 @@
         <v>9</v>
       </c>
       <c r="F112" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G112" t="s">
         <v>17</v>
@@ -3148,7 +3148,7 @@
         <v>9</v>
       </c>
       <c r="F113" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G113" t="s">
         <v>17</v>
@@ -3171,7 +3171,7 @@
         <v>14</v>
       </c>
       <c r="F114" t="n">
-        <v>1870</v>
+        <v>1858</v>
       </c>
       <c r="G114" t="s">
         <v>19</v>
@@ -3194,7 +3194,7 @@
         <v>14</v>
       </c>
       <c r="F115" t="n">
-        <v>1854</v>
+        <v>1815</v>
       </c>
       <c r="G115" t="s">
         <v>18</v>
@@ -3217,7 +3217,7 @@
         <v>14</v>
       </c>
       <c r="F116" t="n">
-        <v>1942</v>
+        <v>1819</v>
       </c>
       <c r="G116" t="s">
         <v>17</v>
@@ -3263,7 +3263,7 @@
         <v>14</v>
       </c>
       <c r="F118" t="n">
-        <v>29</v>
+        <v>2</v>
       </c>
       <c r="G118" t="s">
         <v>17</v>
@@ -3286,7 +3286,7 @@
         <v>9</v>
       </c>
       <c r="F119" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G119" t="s">
         <v>18</v>
@@ -3309,7 +3309,7 @@
         <v>9</v>
       </c>
       <c r="F120" t="n">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="G120" t="s">
         <v>18</v>
@@ -3378,7 +3378,7 @@
         <v>14</v>
       </c>
       <c r="F123" t="n">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="G123" t="s">
         <v>18</v>
@@ -3401,7 +3401,7 @@
         <v>9</v>
       </c>
       <c r="F124" t="n">
-        <v>86</v>
+        <v>100</v>
       </c>
       <c r="G124" t="s">
         <v>19</v>
@@ -3424,7 +3424,7 @@
         <v>9</v>
       </c>
       <c r="F125" t="n">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="G125" t="s">
         <v>19</v>
@@ -3493,7 +3493,7 @@
         <v>14</v>
       </c>
       <c r="F128" t="n">
-        <v>68</v>
+        <v>6</v>
       </c>
       <c r="G128" t="s">
         <v>19</v>
@@ -3516,7 +3516,7 @@
         <v>9</v>
       </c>
       <c r="F129" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G129" t="s">
         <v>22</v>
@@ -3539,7 +3539,7 @@
         <v>9</v>
       </c>
       <c r="F130" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G130" t="s">
         <v>21</v>
@@ -3562,7 +3562,7 @@
         <v>14</v>
       </c>
       <c r="F131" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="G131" t="s">
         <v>21</v>
@@ -3585,7 +3585,7 @@
         <v>14</v>
       </c>
       <c r="F132" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G132" t="s">
         <v>22</v>
@@ -3608,7 +3608,7 @@
         <v>9</v>
       </c>
       <c r="F133" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="G133" t="s">
         <v>39</v>
@@ -3631,7 +3631,7 @@
         <v>9</v>
       </c>
       <c r="F134" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="G134" t="s">
         <v>25</v>
@@ -3677,7 +3677,7 @@
         <v>14</v>
       </c>
       <c r="F136" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="G136" t="s">
         <v>48</v>
@@ -3700,7 +3700,7 @@
         <v>9</v>
       </c>
       <c r="F137" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="G137" t="s">
         <v>42</v>
@@ -3723,7 +3723,7 @@
         <v>9</v>
       </c>
       <c r="F138" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G138" t="s">
         <v>21</v>
@@ -3746,7 +3746,7 @@
         <v>9</v>
       </c>
       <c r="F139" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G139" t="s">
         <v>49</v>
@@ -3792,7 +3792,7 @@
         <v>14</v>
       </c>
       <c r="F141" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G141" t="s">
         <v>21</v>
@@ -3815,7 +3815,7 @@
         <v>9</v>
       </c>
       <c r="F142" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="G142" t="s">
         <v>30</v>
@@ -3861,7 +3861,7 @@
         <v>14</v>
       </c>
       <c r="F144" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G144" t="s">
         <v>30</v>
@@ -3930,7 +3930,7 @@
         <v>9</v>
       </c>
       <c r="F147" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G147" t="s">
         <v>31</v>
@@ -3953,7 +3953,7 @@
         <v>14</v>
       </c>
       <c r="F148" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="G148" t="s">
         <v>31</v>
@@ -3976,7 +3976,7 @@
         <v>9</v>
       </c>
       <c r="F149" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G149" t="s">
         <v>32</v>
@@ -4022,7 +4022,7 @@
         <v>14</v>
       </c>
       <c r="F151" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G151" t="s">
         <v>32</v>
@@ -4045,7 +4045,7 @@
         <v>14</v>
       </c>
       <c r="F152" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G152" t="s">
         <v>32</v>
@@ -4068,7 +4068,7 @@
         <v>9</v>
       </c>
       <c r="F153" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="G153" t="s">
         <v>33</v>
@@ -4137,7 +4137,7 @@
         <v>14</v>
       </c>
       <c r="F156" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G156" t="s">
         <v>33</v>

</xml_diff>